<commit_message>
fix measure, subscale values for an item that was incorrect on the survey
</commit_message>
<xml_diff>
--- a/Phase 1/Track to Treat P1 Codebook.xlsx
+++ b/Phase 1/Track to Treat P1 Codebook.xlsx
@@ -54940,16 +54940,16 @@
         <v>164</v>
       </c>
       <c r="C1012" s="11" t="s">
-        <v>642</v>
+        <v>169</v>
       </c>
       <c r="D1012" s="11">
         <v>32.0</v>
       </c>
       <c r="E1012" s="11" t="s">
-        <v>658</v>
+        <v>169</v>
       </c>
       <c r="F1012" s="11" t="s">
-        <v>659</v>
+        <v>169</v>
       </c>
       <c r="G1012" s="11" t="s">
         <v>167</v>
@@ -55022,16 +55022,16 @@
         <v>648</v>
       </c>
       <c r="C1014" s="11" t="s">
-        <v>642</v>
+        <v>169</v>
       </c>
       <c r="D1014" s="11">
         <v>32.0</v>
       </c>
       <c r="E1014" s="11" t="s">
-        <v>658</v>
+        <v>169</v>
       </c>
       <c r="F1014" s="11" t="s">
-        <v>659</v>
+        <v>169</v>
       </c>
       <c r="G1014" s="11" t="s">
         <v>167</v>
@@ -56308,7 +56308,7 @@
         <v>13</v>
       </c>
       <c r="H1045" s="11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I1045" s="11" t="s">
         <v>168</v>

</xml_diff>